<commit_message>
Se corrigio la planilla de casos de prueba
</commit_message>
<xml_diff>
--- a/Informe Etapa 3/Planilla_Casos_de_Prueba.xlsx
+++ b/Informe Etapa 3/Planilla_Casos_de_Prueba.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matia\Downloads\software\Informe Etapa 3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tarre\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68D4AB80-1E2D-4D0B-9B22-4B6ED85FF341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1797FFF2-EB01-48BF-A047-C4853D927F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Casos de Prueba" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="73">
   <si>
     <t>ID</t>
   </si>
@@ -209,13 +209,43 @@
   </si>
   <si>
     <t>Aprobado</t>
+  </si>
+  <si>
+    <t>El usuario inició sesión correctamente y fue redirigido al dashboard correspondiente según su rol.</t>
+  </si>
+  <si>
+    <t>El sistema impidió el acceso y mostró un mensaje indicando que las credenciales eran incorrectas.</t>
+  </si>
+  <si>
+    <t>El pago fue registrado correctamente y se actualizó el estado de cuenta del residente.</t>
+  </si>
+  <si>
+    <t>El sistema mostró mensajes de validación indicando los campos obligatorios antes de permitir el registro.</t>
+  </si>
+  <si>
+    <t>Se visualizó correctamente el detalle de los pagos, cuotas pendientes y saldo del residente.</t>
+  </si>
+  <si>
+    <t>El historial mostró correctamente todos los pagos realizados por el residente.</t>
+  </si>
+  <si>
+    <t>El sistema generó y descargó correctamente el comprobante de pago en formato PDF.</t>
+  </si>
+  <si>
+    <t>El administrador modificó correctamente la información del pago y los cambios fueron guardados.</t>
+  </si>
+  <si>
+    <t>El sistema cambió correctamente el estado del pago a "Anulado" y actualizó la información correspondiente.</t>
+  </si>
+  <si>
+    <t>El sistema exportó correctamente el reporte de pagos en el formato seleccionado (PDF o Excel).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -230,6 +260,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Inherit"/>
     </font>
   </fonts>
   <fills count="2">
@@ -252,7 +293,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -262,6 +303,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -566,9 +611,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" customWidth="1"/>
+    <col min="7" max="7" width="11.5546875" customWidth="1"/>
+    <col min="8" max="8" width="31.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="28.8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -599,7 +651,7 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="28.8">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -621,14 +673,16 @@
       <c r="G2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="1"/>
+      <c r="H2" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I2" s="1" t="s">
         <v>62</v>
       </c>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="92.4">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -650,14 +704,16 @@
       <c r="G3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="1"/>
+      <c r="H3" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="I3" s="1" t="s">
         <v>62</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="79.2">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
@@ -679,14 +735,16 @@
       <c r="G4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="1"/>
+      <c r="H4" s="5" t="s">
+        <v>65</v>
+      </c>
       <c r="I4" s="1" t="s">
         <v>62</v>
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="105.6">
       <c r="A5" s="1" t="s">
         <v>27</v>
       </c>
@@ -708,14 +766,16 @@
       <c r="G5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="1"/>
+      <c r="H5" s="5" t="s">
+        <v>66</v>
+      </c>
       <c r="I5" s="1" t="s">
         <v>62</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="92.4">
       <c r="A6" s="1" t="s">
         <v>32</v>
       </c>
@@ -735,14 +795,16 @@
       <c r="G6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H6" s="1"/>
+      <c r="H6" s="5" t="s">
+        <v>67</v>
+      </c>
       <c r="I6" s="1" t="s">
         <v>62</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="79.2">
       <c r="A7" s="1" t="s">
         <v>37</v>
       </c>
@@ -762,14 +824,16 @@
       <c r="G7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H7" s="1"/>
+      <c r="H7" s="5" t="s">
+        <v>68</v>
+      </c>
       <c r="I7" s="1" t="s">
         <v>62</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="92.4">
       <c r="A8" s="1" t="s">
         <v>41</v>
       </c>
@@ -789,14 +853,16 @@
       <c r="G8" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="1"/>
+      <c r="H8" s="5" t="s">
+        <v>69</v>
+      </c>
       <c r="I8" s="1" t="s">
         <v>62</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="92.4">
       <c r="A9" s="1" t="s">
         <v>47</v>
       </c>
@@ -816,14 +882,16 @@
       <c r="G9" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="H9" s="1"/>
+      <c r="H9" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="I9" s="1" t="s">
         <v>62</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="105.6">
       <c r="A10" s="1" t="s">
         <v>52</v>
       </c>
@@ -843,14 +911,16 @@
       <c r="G10" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="1"/>
+      <c r="H10" s="5" t="s">
+        <v>71</v>
+      </c>
       <c r="I10" s="1" t="s">
         <v>62</v>
       </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="92.4">
       <c r="A11" s="1" t="s">
         <v>56</v>
       </c>
@@ -872,14 +942,16 @@
       <c r="G11" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="H11" s="1"/>
+      <c r="H11" s="5" t="s">
+        <v>72</v>
+      </c>
       <c r="I11" s="1" t="s">
         <v>62</v>
       </c>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>

</xml_diff>